<commit_message>
Added My Daily Routine Excel && Added Python Code for the Formula && Added My Record Maintaincace File
</commit_message>
<xml_diff>
--- a/Python Daily Workflow Stats.xlsx
+++ b/Python Daily Workflow Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GiTCloneE\PythonRepo\LPU-PYTHON\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7BB516B-66DD-4061-A060-70078E78391D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D89422-4117-42B8-8AE7-77566545DADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="22284" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="22308" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Routine Data" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
   <si>
     <t>Date</t>
   </si>
@@ -208,6 +208,9 @@
   </si>
   <si>
     <t>Bhuvanagiri Gireesh</t>
+  </si>
+  <si>
+    <t>Column Total</t>
   </si>
 </sst>
 </file>
@@ -217,7 +220,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -261,8 +264,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -290,6 +301,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1" tint="0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -336,19 +353,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -359,6 +369,19 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -642,7 +665,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4567193D-5B77-445E-92C2-4710E5F613D2}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.77734375" customWidth="1"/>
@@ -660,56 +683,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
       <c r="E2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="11">
         <v>12627043</v>
       </c>
-      <c r="G2" s="6"/>
+      <c r="G2" s="11"/>
     </row>
     <row r="3" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
       <c r="E3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="G3" s="9"/>
     </row>
     <row r="4" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
@@ -730,51 +753,51 @@
       <c r="N4" s="7"/>
     </row>
     <row r="5" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="9" t="s">
+      <c r="A5" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="9" t="s">
+      <c r="E5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="K5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="L5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="M5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N5" s="9" t="s">
+      <c r="N5" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
+      <c r="A6" s="3">
         <v>46247</v>
       </c>
       <c r="B6" s="1">
@@ -798,11 +821,11 @@
       <c r="H6" s="1">
         <v>90</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="6">
         <f t="shared" ref="I6:I45" si="0">IF(COUNTA(B6:H6)=0,"",SUM(B6:F6,H6))</f>
         <v>900</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="6">
         <f t="shared" ref="J6:J45" si="1">IF(I6="","",1440-I6)</f>
         <v>540</v>
       </c>
@@ -815,12 +838,12 @@
       <c r="M6" s="1">
         <v>5</v>
       </c>
-      <c r="N6" s="10" t="s">
+      <c r="N6" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8">
+      <c r="A7" s="3">
         <v>46248</v>
       </c>
       <c r="B7" s="1">
@@ -844,11 +867,11 @@
       <c r="H7" s="1">
         <v>40</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="6">
         <f t="shared" si="0"/>
         <v>820</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="6">
         <f t="shared" si="1"/>
         <v>620</v>
       </c>
@@ -861,12 +884,12 @@
       <c r="M7" s="1">
         <v>5</v>
       </c>
-      <c r="N7" s="10" t="s">
+      <c r="N7" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+      <c r="A8" s="3">
         <v>46249</v>
       </c>
       <c r="B8" s="1">
@@ -890,11 +913,11 @@
       <c r="H8" s="1">
         <v>120</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="6">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="6">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
@@ -907,12 +930,12 @@
       <c r="M8" s="1">
         <v>4</v>
       </c>
-      <c r="N8" s="10" t="s">
+      <c r="N8" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8">
+      <c r="A9" s="3">
         <v>46250</v>
       </c>
       <c r="B9" s="1">
@@ -936,11 +959,11 @@
       <c r="H9" s="1">
         <v>120</v>
       </c>
-      <c r="I9" s="11">
+      <c r="I9" s="6">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="6">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
@@ -953,12 +976,12 @@
       <c r="M9" s="1">
         <v>5</v>
       </c>
-      <c r="N9" s="10" t="s">
+      <c r="N9" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8">
+      <c r="A10" s="3">
         <v>46251</v>
       </c>
       <c r="B10" s="1">
@@ -982,11 +1005,11 @@
       <c r="H10" s="1">
         <v>60</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="6">
         <f t="shared" si="0"/>
         <v>885</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="6">
         <f t="shared" si="1"/>
         <v>555</v>
       </c>
@@ -999,12 +1022,12 @@
       <c r="M10" s="1">
         <v>5</v>
       </c>
-      <c r="N10" s="10" t="s">
+      <c r="N10" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8">
+      <c r="A11" s="3">
         <v>46252</v>
       </c>
       <c r="B11" s="1">
@@ -1028,11 +1051,11 @@
       <c r="H11" s="1">
         <v>60</v>
       </c>
-      <c r="I11" s="11">
+      <c r="I11" s="6">
         <f t="shared" si="0"/>
         <v>915</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="6">
         <f t="shared" si="1"/>
         <v>525</v>
       </c>
@@ -1045,12 +1068,12 @@
       <c r="M11" s="1">
         <v>5</v>
       </c>
-      <c r="N11" s="10" t="s">
+      <c r="N11" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8">
+      <c r="A12" s="3">
         <v>46253</v>
       </c>
       <c r="B12" s="1">
@@ -1074,11 +1097,11 @@
       <c r="H12" s="1">
         <v>90</v>
       </c>
-      <c r="I12" s="11">
+      <c r="I12" s="6">
         <f t="shared" si="0"/>
         <v>880</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="6">
         <f t="shared" si="1"/>
         <v>560</v>
       </c>
@@ -1091,12 +1114,12 @@
       <c r="M12" s="1">
         <v>5</v>
       </c>
-      <c r="N12" s="10" t="s">
+      <c r="N12" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8">
+      <c r="A13" s="3">
         <v>46254</v>
       </c>
       <c r="B13" s="1">
@@ -1120,11 +1143,11 @@
       <c r="H13" s="1">
         <v>90</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="6">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="6">
         <f t="shared" si="1"/>
         <v>540</v>
       </c>
@@ -1137,12 +1160,12 @@
       <c r="M13" s="1">
         <v>4</v>
       </c>
-      <c r="N13" s="10" t="s">
+      <c r="N13" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8">
+      <c r="A14" s="3">
         <v>46255</v>
       </c>
       <c r="B14" s="1">
@@ -1166,11 +1189,11 @@
       <c r="H14" s="1">
         <v>40</v>
       </c>
-      <c r="I14" s="11">
+      <c r="I14" s="6">
         <f t="shared" si="0"/>
         <v>820</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="6">
         <f t="shared" si="1"/>
         <v>620</v>
       </c>
@@ -1183,12 +1206,12 @@
       <c r="M14" s="1">
         <v>5</v>
       </c>
-      <c r="N14" s="10" t="s">
+      <c r="N14" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="8">
+      <c r="A15" s="3">
         <v>46256</v>
       </c>
       <c r="B15" s="1">
@@ -1212,11 +1235,11 @@
       <c r="H15" s="1">
         <v>120</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="6">
         <f t="shared" si="0"/>
         <v>720</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="6">
         <f t="shared" si="1"/>
         <v>720</v>
       </c>
@@ -1229,12 +1252,12 @@
       <c r="M15" s="1">
         <v>5</v>
       </c>
-      <c r="N15" s="10" t="s">
+      <c r="N15" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="8">
+      <c r="A16" s="3">
         <v>46257</v>
       </c>
       <c r="B16" s="1">
@@ -1258,11 +1281,11 @@
       <c r="H16" s="1">
         <v>120</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="6">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="6">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
@@ -1275,12 +1298,12 @@
       <c r="M16" s="1">
         <v>4</v>
       </c>
-      <c r="N16" s="10" t="s">
+      <c r="N16" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8">
+      <c r="A17" s="3">
         <v>46258</v>
       </c>
       <c r="B17" s="1">
@@ -1304,11 +1327,11 @@
       <c r="H17" s="1">
         <v>60</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17" s="6">
         <f t="shared" si="0"/>
         <v>885</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17" s="6">
         <f t="shared" si="1"/>
         <v>555</v>
       </c>
@@ -1321,12 +1344,12 @@
       <c r="M17" s="1">
         <v>5</v>
       </c>
-      <c r="N17" s="10" t="s">
+      <c r="N17" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8">
+      <c r="A18" s="3">
         <v>46259</v>
       </c>
       <c r="B18" s="1">
@@ -1350,11 +1373,11 @@
       <c r="H18" s="1">
         <v>60</v>
       </c>
-      <c r="I18" s="11">
+      <c r="I18" s="6">
         <f t="shared" si="0"/>
         <v>915</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="6">
         <f t="shared" si="1"/>
         <v>525</v>
       </c>
@@ -1367,12 +1390,12 @@
       <c r="M18" s="1">
         <v>4</v>
       </c>
-      <c r="N18" s="10" t="s">
+      <c r="N18" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8">
+      <c r="A19" s="3">
         <v>46260</v>
       </c>
       <c r="B19" s="1">
@@ -1396,11 +1419,11 @@
       <c r="H19" s="1">
         <v>90</v>
       </c>
-      <c r="I19" s="11">
+      <c r="I19" s="6">
         <f t="shared" si="0"/>
         <v>880</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="6">
         <f t="shared" si="1"/>
         <v>560</v>
       </c>
@@ -1413,12 +1436,12 @@
       <c r="M19" s="1">
         <v>5</v>
       </c>
-      <c r="N19" s="10" t="s">
+      <c r="N19" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8">
+      <c r="A20" s="3">
         <v>46261</v>
       </c>
       <c r="B20" s="1">
@@ -1442,11 +1465,11 @@
       <c r="H20" s="1">
         <v>90</v>
       </c>
-      <c r="I20" s="11">
+      <c r="I20" s="6">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20" s="6">
         <f t="shared" si="1"/>
         <v>540</v>
       </c>
@@ -1459,12 +1482,12 @@
       <c r="M20" s="1">
         <v>5</v>
       </c>
-      <c r="N20" s="10" t="s">
+      <c r="N20" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="8">
+      <c r="A21" s="3">
         <v>46262</v>
       </c>
       <c r="B21" s="1">
@@ -1488,11 +1511,11 @@
       <c r="H21" s="1">
         <v>40</v>
       </c>
-      <c r="I21" s="11">
+      <c r="I21" s="6">
         <f t="shared" si="0"/>
         <v>820</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21" s="6">
         <f t="shared" si="1"/>
         <v>620</v>
       </c>
@@ -1505,12 +1528,12 @@
       <c r="M21" s="1">
         <v>5</v>
       </c>
-      <c r="N21" s="10" t="s">
+      <c r="N21" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="8">
+      <c r="A22" s="3">
         <v>46263</v>
       </c>
       <c r="B22" s="1">
@@ -1534,11 +1557,11 @@
       <c r="H22" s="1">
         <v>120</v>
       </c>
-      <c r="I22" s="11">
+      <c r="I22" s="6">
         <f t="shared" si="0"/>
         <v>720</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22" s="6">
         <f t="shared" si="1"/>
         <v>720</v>
       </c>
@@ -1551,12 +1574,12 @@
       <c r="M22" s="1">
         <v>4</v>
       </c>
-      <c r="N22" s="10" t="s">
+      <c r="N22" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="8">
+      <c r="A23" s="3">
         <v>46264</v>
       </c>
       <c r="B23" s="1">
@@ -1580,11 +1603,11 @@
       <c r="H23" s="1">
         <v>120</v>
       </c>
-      <c r="I23" s="11">
+      <c r="I23" s="6">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23" s="6">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
@@ -1597,12 +1620,12 @@
       <c r="M23" s="1">
         <v>5</v>
       </c>
-      <c r="N23" s="10" t="s">
+      <c r="N23" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="8">
+      <c r="A24" s="3">
         <v>46265</v>
       </c>
       <c r="B24" s="1">
@@ -1626,11 +1649,11 @@
       <c r="H24" s="1">
         <v>60</v>
       </c>
-      <c r="I24" s="11">
+      <c r="I24" s="6">
         <f t="shared" si="0"/>
         <v>915</v>
       </c>
-      <c r="J24" s="11">
+      <c r="J24" s="6">
         <f t="shared" si="1"/>
         <v>525</v>
       </c>
@@ -1643,12 +1666,12 @@
       <c r="M24" s="1">
         <v>5</v>
       </c>
-      <c r="N24" s="10" t="s">
+      <c r="N24" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="8">
+      <c r="A25" s="3">
         <v>46266</v>
       </c>
       <c r="B25" s="1">
@@ -1672,11 +1695,11 @@
       <c r="H25" s="1">
         <v>90</v>
       </c>
-      <c r="I25" s="11">
+      <c r="I25" s="6">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25" s="6">
         <f t="shared" si="1"/>
         <v>540</v>
       </c>
@@ -1689,12 +1712,12 @@
       <c r="M25" s="1">
         <v>5</v>
       </c>
-      <c r="N25" s="10" t="s">
+      <c r="N25" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="8">
+      <c r="A26" s="3">
         <v>46267</v>
       </c>
       <c r="B26" s="1">
@@ -1718,11 +1741,11 @@
       <c r="H26" s="1">
         <v>90</v>
       </c>
-      <c r="I26" s="11">
+      <c r="I26" s="6">
         <f t="shared" si="0"/>
         <v>880</v>
       </c>
-      <c r="J26" s="11">
+      <c r="J26" s="6">
         <f t="shared" si="1"/>
         <v>560</v>
       </c>
@@ -1735,12 +1758,12 @@
       <c r="M26" s="1">
         <v>5</v>
       </c>
-      <c r="N26" s="10" t="s">
+      <c r="N26" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="8">
+      <c r="A27" s="3">
         <v>46268</v>
       </c>
       <c r="B27" s="1">
@@ -1764,11 +1787,11 @@
       <c r="H27" s="1">
         <v>90</v>
       </c>
-      <c r="I27" s="11">
+      <c r="I27" s="6">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J27" s="6">
         <f t="shared" si="1"/>
         <v>540</v>
       </c>
@@ -1781,12 +1804,12 @@
       <c r="M27" s="1">
         <v>4</v>
       </c>
-      <c r="N27" s="10" t="s">
+      <c r="N27" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8">
+      <c r="A28" s="3">
         <v>46269</v>
       </c>
       <c r="B28" s="1">
@@ -1810,11 +1833,11 @@
       <c r="H28" s="1">
         <v>60</v>
       </c>
-      <c r="I28" s="11">
+      <c r="I28" s="6">
         <f t="shared" si="0"/>
         <v>885</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J28" s="6">
         <f t="shared" si="1"/>
         <v>555</v>
       </c>
@@ -1827,12 +1850,12 @@
       <c r="M28" s="1">
         <v>5</v>
       </c>
-      <c r="N28" s="10" t="s">
+      <c r="N28" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="8">
+      <c r="A29" s="3">
         <v>46270</v>
       </c>
       <c r="B29" s="1">
@@ -1856,11 +1879,11 @@
       <c r="H29" s="1">
         <v>90</v>
       </c>
-      <c r="I29" s="11">
+      <c r="I29" s="6">
         <f t="shared" si="0"/>
         <v>945</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29" s="6">
         <f t="shared" si="1"/>
         <v>495</v>
       </c>
@@ -1873,12 +1896,12 @@
       <c r="M29" s="1">
         <v>5</v>
       </c>
-      <c r="N29" s="10" t="s">
+      <c r="N29" s="5" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="8">
+      <c r="A30" s="3">
         <v>46271</v>
       </c>
       <c r="B30" s="1">
@@ -1902,11 +1925,11 @@
       <c r="H30" s="1">
         <v>120</v>
       </c>
-      <c r="I30" s="11">
+      <c r="I30" s="6">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30" s="6">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
@@ -1919,12 +1942,12 @@
       <c r="M30" s="1">
         <v>5</v>
       </c>
-      <c r="N30" s="10" t="s">
+      <c r="N30" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="8">
+      <c r="A31" s="3">
         <v>46272</v>
       </c>
       <c r="B31" s="1">
@@ -1948,11 +1971,11 @@
       <c r="H31" s="1">
         <v>60</v>
       </c>
-      <c r="I31" s="11">
+      <c r="I31" s="6">
         <f t="shared" si="0"/>
         <v>885</v>
       </c>
-      <c r="J31" s="11">
+      <c r="J31" s="6">
         <f t="shared" si="1"/>
         <v>555</v>
       </c>
@@ -1965,12 +1988,12 @@
       <c r="M31" s="1">
         <v>5</v>
       </c>
-      <c r="N31" s="10" t="s">
+      <c r="N31" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="8">
+      <c r="A32" s="3">
         <v>46273</v>
       </c>
       <c r="B32" s="1">
@@ -1994,11 +2017,11 @@
       <c r="H32" s="1">
         <v>90</v>
       </c>
-      <c r="I32" s="11">
+      <c r="I32" s="6">
         <f t="shared" si="0"/>
         <v>940</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32" s="6">
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
@@ -2011,12 +2034,12 @@
       <c r="M32" s="1">
         <v>5</v>
       </c>
-      <c r="N32" s="10" t="s">
+      <c r="N32" s="5" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="8">
+      <c r="A33" s="3">
         <v>46274</v>
       </c>
       <c r="B33" s="1">
@@ -2040,11 +2063,11 @@
       <c r="H33" s="1">
         <v>60</v>
       </c>
-      <c r="I33" s="11">
+      <c r="I33" s="6">
         <f t="shared" si="0"/>
         <v>870</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33" s="6">
         <f t="shared" si="1"/>
         <v>570</v>
       </c>
@@ -2057,12 +2080,12 @@
       <c r="M33" s="1">
         <v>5</v>
       </c>
-      <c r="N33" s="10" t="s">
+      <c r="N33" s="5" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8">
+      <c r="A34" s="3">
         <v>46275</v>
       </c>
       <c r="B34" s="1">
@@ -2086,11 +2109,11 @@
       <c r="H34" s="1">
         <v>90</v>
       </c>
-      <c r="I34" s="11">
+      <c r="I34" s="6">
         <f t="shared" si="0"/>
         <v>945</v>
       </c>
-      <c r="J34" s="11">
+      <c r="J34" s="6">
         <f t="shared" si="1"/>
         <v>495</v>
       </c>
@@ -2103,12 +2126,12 @@
       <c r="M34" s="1">
         <v>5</v>
       </c>
-      <c r="N34" s="10" t="s">
+      <c r="N34" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="8">
+      <c r="A35" s="3">
         <v>46276</v>
       </c>
       <c r="B35" s="1">
@@ -2132,11 +2155,11 @@
       <c r="H35" s="1">
         <v>40</v>
       </c>
-      <c r="I35" s="11">
+      <c r="I35" s="6">
         <f t="shared" si="0"/>
         <v>820</v>
       </c>
-      <c r="J35" s="11">
+      <c r="J35" s="6">
         <f t="shared" si="1"/>
         <v>620</v>
       </c>
@@ -2149,12 +2172,12 @@
       <c r="M35" s="1">
         <v>4</v>
       </c>
-      <c r="N35" s="10" t="s">
+      <c r="N35" s="5" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="8">
+      <c r="A36" s="3">
         <v>46277</v>
       </c>
       <c r="B36" s="1">
@@ -2178,11 +2201,11 @@
       <c r="H36" s="1">
         <v>90</v>
       </c>
-      <c r="I36" s="11">
+      <c r="I36" s="6">
         <f t="shared" si="0"/>
         <v>930</v>
       </c>
-      <c r="J36" s="11">
+      <c r="J36" s="6">
         <f t="shared" si="1"/>
         <v>510</v>
       </c>
@@ -2195,12 +2218,12 @@
       <c r="M36" s="1">
         <v>5</v>
       </c>
-      <c r="N36" s="10" t="s">
+      <c r="N36" s="5" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8">
+      <c r="A37" s="3">
         <v>46278</v>
       </c>
       <c r="B37" s="1">
@@ -2224,11 +2247,11 @@
       <c r="H37" s="1">
         <v>120</v>
       </c>
-      <c r="I37" s="11">
+      <c r="I37" s="6">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
-      <c r="J37" s="11">
+      <c r="J37" s="6">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
@@ -2241,12 +2264,12 @@
       <c r="M37" s="1">
         <v>5</v>
       </c>
-      <c r="N37" s="10" t="s">
+      <c r="N37" s="5" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8">
+      <c r="A38" s="3">
         <v>46279</v>
       </c>
       <c r="B38" s="1">
@@ -2270,11 +2293,11 @@
       <c r="H38" s="1">
         <v>60</v>
       </c>
-      <c r="I38" s="11">
+      <c r="I38" s="6">
         <f t="shared" si="0"/>
         <v>915</v>
       </c>
-      <c r="J38" s="11">
+      <c r="J38" s="6">
         <f t="shared" si="1"/>
         <v>525</v>
       </c>
@@ -2287,12 +2310,12 @@
       <c r="M38" s="1">
         <v>5</v>
       </c>
-      <c r="N38" s="10" t="s">
+      <c r="N38" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="8">
+      <c r="A39" s="3">
         <v>46280</v>
       </c>
       <c r="B39" s="1">
@@ -2316,11 +2339,11 @@
       <c r="H39" s="1">
         <v>90</v>
       </c>
-      <c r="I39" s="11">
+      <c r="I39" s="6">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="J39" s="11">
+      <c r="J39" s="6">
         <f t="shared" si="1"/>
         <v>540</v>
       </c>
@@ -2333,12 +2356,12 @@
       <c r="M39" s="1">
         <v>5</v>
       </c>
-      <c r="N39" s="10" t="s">
+      <c r="N39" s="5" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="8">
+      <c r="A40" s="3">
         <v>46281</v>
       </c>
       <c r="B40" s="1">
@@ -2362,11 +2385,11 @@
       <c r="H40" s="1">
         <v>60</v>
       </c>
-      <c r="I40" s="11">
+      <c r="I40" s="6">
         <f t="shared" si="0"/>
         <v>925</v>
       </c>
-      <c r="J40" s="11">
+      <c r="J40" s="6">
         <f t="shared" si="1"/>
         <v>515</v>
       </c>
@@ -2379,12 +2402,12 @@
       <c r="M40" s="1">
         <v>5</v>
       </c>
-      <c r="N40" s="10" t="s">
+      <c r="N40" s="5" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="8">
+      <c r="A41" s="3">
         <v>46282</v>
       </c>
       <c r="B41" s="1">
@@ -2408,11 +2431,11 @@
       <c r="H41" s="1">
         <v>90</v>
       </c>
-      <c r="I41" s="11">
+      <c r="I41" s="6">
         <f t="shared" si="0"/>
         <v>900</v>
       </c>
-      <c r="J41" s="11">
+      <c r="J41" s="6">
         <f t="shared" si="1"/>
         <v>540</v>
       </c>
@@ -2425,12 +2448,12 @@
       <c r="M41" s="1">
         <v>4</v>
       </c>
-      <c r="N41" s="10" t="s">
+      <c r="N41" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="8">
+      <c r="A42" s="3">
         <v>46283</v>
       </c>
       <c r="B42" s="1">
@@ -2454,11 +2477,11 @@
       <c r="H42" s="1">
         <v>60</v>
       </c>
-      <c r="I42" s="11">
+      <c r="I42" s="6">
         <f t="shared" si="0"/>
         <v>885</v>
       </c>
-      <c r="J42" s="11">
+      <c r="J42" s="6">
         <f t="shared" si="1"/>
         <v>555</v>
       </c>
@@ -2471,12 +2494,12 @@
       <c r="M42" s="1">
         <v>5</v>
       </c>
-      <c r="N42" s="10" t="s">
+      <c r="N42" s="5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="8">
+      <c r="A43" s="3">
         <v>46284</v>
       </c>
       <c r="B43" s="1">
@@ -2500,11 +2523,11 @@
       <c r="H43" s="1">
         <v>90</v>
       </c>
-      <c r="I43" s="11">
+      <c r="I43" s="6">
         <f t="shared" si="0"/>
         <v>945</v>
       </c>
-      <c r="J43" s="11">
+      <c r="J43" s="6">
         <f t="shared" si="1"/>
         <v>495</v>
       </c>
@@ -2517,12 +2540,12 @@
       <c r="M43" s="1">
         <v>5</v>
       </c>
-      <c r="N43" s="10" t="s">
+      <c r="N43" s="5" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="8">
+      <c r="A44" s="3">
         <v>46285</v>
       </c>
       <c r="B44" s="1">
@@ -2546,11 +2569,11 @@
       <c r="H44" s="1">
         <v>120</v>
       </c>
-      <c r="I44" s="11">
+      <c r="I44" s="6">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
-      <c r="J44" s="11">
+      <c r="J44" s="6">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
@@ -2563,12 +2586,12 @@
       <c r="M44" s="1">
         <v>4</v>
       </c>
-      <c r="N44" s="10" t="s">
+      <c r="N44" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="8">
+      <c r="A45" s="3">
         <v>46286</v>
       </c>
       <c r="B45" s="1">
@@ -2592,11 +2615,11 @@
       <c r="H45" s="1">
         <v>60</v>
       </c>
-      <c r="I45" s="11">
+      <c r="I45" s="6">
         <f t="shared" si="0"/>
         <v>915</v>
       </c>
-      <c r="J45" s="11">
+      <c r="J45" s="6">
         <f t="shared" si="1"/>
         <v>525</v>
       </c>
@@ -2609,8 +2632,61 @@
       <c r="M45" s="1">
         <v>5</v>
       </c>
-      <c r="N45" s="10" t="s">
+      <c r="N45" s="5" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" s="13">
+        <f>SUM(B6:B45)</f>
+        <v>16080</v>
+      </c>
+      <c r="C46" s="13">
+        <f>SUM(C6:C45)</f>
+        <v>1100</v>
+      </c>
+      <c r="D46" s="13">
+        <f t="shared" ref="D46:M46" si="2">SUM(D6:D45)</f>
+        <v>3960</v>
+      </c>
+      <c r="E46" s="13">
+        <f t="shared" si="2"/>
+        <v>1530</v>
+      </c>
+      <c r="F46" s="13">
+        <f t="shared" si="2"/>
+        <v>8640</v>
+      </c>
+      <c r="G46" s="13">
+        <f t="shared" si="2"/>
+        <v>144</v>
+      </c>
+      <c r="H46" s="13">
+        <f t="shared" si="2"/>
+        <v>3310</v>
+      </c>
+      <c r="I46" s="13">
+        <f t="shared" si="2"/>
+        <v>34620</v>
+      </c>
+      <c r="J46" s="13">
+        <f t="shared" si="2"/>
+        <v>22980</v>
+      </c>
+      <c r="K46" s="13">
+        <f>AVERAGE(K6:K45)</f>
+        <v>4.5</v>
+      </c>
+      <c r="L46" s="13">
+        <f>AVERAGE(L6:L45)</f>
+        <v>4.55</v>
+      </c>
+      <c r="M46" s="13">
+        <f>AVERAGE(M6:M45)</f>
+        <v>4.7750000000000004</v>
       </c>
     </row>
   </sheetData>
@@ -2624,5 +2700,6 @@
     <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added CAP776-Minor Report As PDF && WordFile Converted Into PDF, Deleted respective WordFiles
</commit_message>
<xml_diff>
--- a/Python Daily Workflow Stats.xlsx
+++ b/Python Daily Workflow Stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GiTCloneE\PythonRepo\LPU-PYTHON\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D89422-4117-42B8-8AE7-77566545DADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{603101B2-9A18-4A25-B50C-D8AF93091CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="22308" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
   <si>
     <t>Date</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>Column Total</t>
+  </si>
+  <si>
+    <t>Average</t>
   </si>
 </sst>
 </file>
@@ -220,7 +223,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,8 +275,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -307,6 +318,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -353,7 +370,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -371,6 +388,12 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -378,11 +401,11 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -665,7 +688,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4567193D-5B77-445E-92C2-4710E5F613D2}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.77734375" customWidth="1"/>
@@ -683,74 +706,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
       <c r="E2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="11">
+      <c r="F2" s="13">
         <v>12627043</v>
       </c>
-      <c r="G2" s="11"/>
+      <c r="G2" s="13"/>
     </row>
     <row r="3" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
       <c r="E3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="9"/>
+      <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
     </row>
     <row r="5" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -2637,56 +2660,94 @@
       </c>
     </row>
     <row r="46" spans="1:14" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B46" s="13">
+      <c r="A46" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" s="8">
         <f>SUM(B6:B45)</f>
         <v>16080</v>
       </c>
-      <c r="C46" s="13">
+      <c r="C46" s="8">
         <f>SUM(C6:C45)</f>
         <v>1100</v>
       </c>
-      <c r="D46" s="13">
-        <f t="shared" ref="D46:M46" si="2">SUM(D6:D45)</f>
+      <c r="D46" s="8">
+        <f t="shared" ref="D46:J46" si="2">SUM(D6:D45)</f>
         <v>3960</v>
       </c>
-      <c r="E46" s="13">
+      <c r="E46" s="8">
         <f t="shared" si="2"/>
         <v>1530</v>
       </c>
-      <c r="F46" s="13">
+      <c r="F46" s="8">
         <f t="shared" si="2"/>
         <v>8640</v>
       </c>
-      <c r="G46" s="13">
+      <c r="G46" s="8">
         <f t="shared" si="2"/>
         <v>144</v>
       </c>
-      <c r="H46" s="13">
+      <c r="H46" s="8">
         <f t="shared" si="2"/>
         <v>3310</v>
       </c>
-      <c r="I46" s="13">
+      <c r="I46" s="8">
         <f t="shared" si="2"/>
         <v>34620</v>
       </c>
-      <c r="J46" s="13">
+      <c r="J46" s="8">
         <f t="shared" si="2"/>
         <v>22980</v>
       </c>
-      <c r="K46" s="13">
+      <c r="K46" s="8">
         <f>AVERAGE(K6:K45)</f>
         <v>4.5</v>
       </c>
-      <c r="L46" s="13">
+      <c r="L46" s="8">
         <f>AVERAGE(L6:L45)</f>
         <v>4.55</v>
       </c>
-      <c r="M46" s="13">
+      <c r="M46" s="8">
         <f>AVERAGE(M6:M45)</f>
         <v>4.7750000000000004</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B47" s="15">
+        <f>AVERAGE(B6:B45)</f>
+        <v>402</v>
+      </c>
+      <c r="C47" s="15">
+        <f t="shared" ref="C47:J47" si="3">AVERAGE(C6:C45)</f>
+        <v>27.5</v>
+      </c>
+      <c r="D47" s="15">
+        <f t="shared" si="3"/>
+        <v>99</v>
+      </c>
+      <c r="E47" s="15">
+        <f t="shared" si="3"/>
+        <v>38.25</v>
+      </c>
+      <c r="F47" s="15">
+        <f t="shared" si="3"/>
+        <v>216</v>
+      </c>
+      <c r="G47" s="15">
+        <f t="shared" si="3"/>
+        <v>3.6</v>
+      </c>
+      <c r="H47" s="15">
+        <f t="shared" si="3"/>
+        <v>82.75</v>
+      </c>
+      <c r="I47" s="15"/>
+      <c r="J47" s="15">
+        <f t="shared" si="3"/>
+        <v>574.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>